<commit_message>
Adjusted shutdown so that in new dev boards, flag BOARD_HAS_BATT_DISCONNECT will allow shutdown to properly turn BATT_SW_Enable to high z and disconnect battery
</commit_message>
<xml_diff>
--- a/Docs/SRS Opcodes.xlsx
+++ b/Docs/SRS Opcodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\data\0_grants\0_HORNET\0-SW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexbaldwin/Desktop/GitHub Repos/OpenNerve-Implantable-Pulse-Generator/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20ED4D7B-CE61-4D21-ACB3-2AC140828690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="7" activeTab="12" xr2:uid="{60045939-FD78-43B2-9714-F2E4455A8B87}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" firstSheet="7" activeTab="12" xr2:uid="{60045939-FD78-43B2-9714-F2E4455A8B87}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="5" r:id="rId1"/>
@@ -1494,6 +1494,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1504,9 +1516,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1598,15 +1607,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1943,37 +1943,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1045C550-E246-4B88-8A9D-FF0ABB166E69}">
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.23046875" customWidth="1"/>
-    <col min="2" max="2" width="7.15234375" customWidth="1"/>
-    <col min="3" max="3" width="5.61328125" customWidth="1"/>
+    <col min="1" max="1" width="27.1640625" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" customWidth="1"/>
     <col min="4" max="4" width="33" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.15234375" customWidth="1"/>
-    <col min="8" max="8" width="7.15234375" customWidth="1"/>
-    <col min="9" max="9" width="38.61328125" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.1640625" customWidth="1"/>
+    <col min="8" max="8" width="7.1640625" customWidth="1"/>
+    <col min="9" max="9" width="38.6640625" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="9"/>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="31" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="33"/>
-    </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="37"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>185</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
         <v>182</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
         <v>183</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>184</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>171</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>172</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>180</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>181</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>267</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>173</v>
       </c>
@@ -2293,7 +2293,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>178</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="64" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A13" s="26" t="s">
         <v>239</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="H15" s="29">
         <v>0</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="H16" s="29">
         <v>1</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.2">
       <c r="H17" t="s">
         <v>259</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.2">
       <c r="H18" t="s">
         <v>261</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="8:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="8:9" x14ac:dyDescent="0.2">
       <c r="H19" t="s">
         <v>263</v>
       </c>
@@ -2397,7 +2397,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="20" spans="8:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="8:9" x14ac:dyDescent="0.2">
       <c r="H20" t="s">
         <v>265</v>
       </c>
@@ -2418,57 +2418,57 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C45638A-5C24-4BBF-B99C-EFB2214A1DEA}">
   <dimension ref="A1:O3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.23046875" customWidth="1"/>
-    <col min="3" max="8" width="13.765625" customWidth="1"/>
-    <col min="9" max="9" width="15.765625" customWidth="1"/>
-    <col min="10" max="10" width="10.4609375" customWidth="1"/>
-    <col min="11" max="11" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.15234375" customWidth="1"/>
-    <col min="13" max="13" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.23046875" customWidth="1"/>
-    <col min="15" max="15" width="9.4609375" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.1640625" customWidth="1"/>
+    <col min="3" max="8" width="13.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.5" customWidth="1"/>
+    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1640625" customWidth="1"/>
+    <col min="13" max="13" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.1640625" customWidth="1"/>
+    <col min="15" max="15" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="35" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="37"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="40"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="41" t="s">
         <v>162</v>
       </c>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="40"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="43"/>
       <c r="J2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>158</v>
       </c>
@@ -2549,40 +2549,40 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30815585-3AA0-4CBE-987F-949816EFA506}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.23046875" customWidth="1"/>
-    <col min="2" max="2" width="5.765625" customWidth="1"/>
-    <col min="3" max="3" width="5.15234375" customWidth="1"/>
-    <col min="4" max="4" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.23046875" customWidth="1"/>
+    <col min="1" max="1" width="6.1640625" customWidth="1"/>
+    <col min="2" max="2" width="5.83203125" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1640625" customWidth="1"/>
     <col min="6" max="6" width="5" customWidth="1"/>
-    <col min="7" max="7" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="8" max="13" width="14.3828125" customWidth="1"/>
-    <col min="14" max="14" width="10.15234375" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="13" width="14.33203125" customWidth="1"/>
+    <col min="14" max="14" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="35" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="37"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="40"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2604,19 +2604,19 @@
       <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="35" t="s">
+      <c r="H2" s="38" t="s">
         <v>166</v>
       </c>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="37"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="40"/>
       <c r="N2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>164</v>
       </c>
@@ -2660,7 +2660,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>293</v>
       </c>
@@ -2679,58 +2679,58 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{733B885E-75D9-45E5-8D2B-75991212B440}">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.765625" customWidth="1"/>
-    <col min="2" max="2" width="5.4609375" customWidth="1"/>
-    <col min="3" max="3" width="12.765625" customWidth="1"/>
-    <col min="4" max="4" width="14.765625" customWidth="1"/>
-    <col min="5" max="5" width="13.3828125" customWidth="1"/>
-    <col min="6" max="6" width="14.765625" customWidth="1"/>
-    <col min="7" max="7" width="12.765625" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="5.5" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="9.84375" customWidth="1"/>
-    <col min="10" max="10" width="5.23046875" customWidth="1"/>
-    <col min="11" max="11" width="4.15234375" customWidth="1"/>
-    <col min="12" max="12" width="6.23046875" customWidth="1"/>
-    <col min="14" max="14" width="9.84375" customWidth="1"/>
+    <col min="9" max="9" width="9.83203125" customWidth="1"/>
+    <col min="10" max="10" width="5.1640625" customWidth="1"/>
+    <col min="11" max="11" width="4.1640625" customWidth="1"/>
+    <col min="12" max="12" width="6.1640625" customWidth="1"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A1" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="35" t="s">
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="37"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="40"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="41" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="40"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="43"/>
       <c r="I2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>167</v>
       </c>
@@ -2794,7 +2794,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>294</v>
       </c>
@@ -2813,43 +2813,43 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B271A376-0C1B-4C38-8AE4-CB714D2B3429}">
   <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.3828125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.69140625" customWidth="1"/>
-    <col min="4" max="4" width="10.4609375" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="14.61328125" customWidth="1"/>
-    <col min="7" max="7" width="12.3828125" customWidth="1"/>
-    <col min="8" max="8" width="6.23046875" customWidth="1"/>
-    <col min="9" max="9" width="7.765625" customWidth="1"/>
-    <col min="10" max="10" width="3.84375" customWidth="1"/>
-    <col min="11" max="11" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="31.765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" customWidth="1"/>
+    <col min="4" max="4" width="10.5" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" customWidth="1"/>
+    <col min="10" max="10" width="3.83203125" customWidth="1"/>
+    <col min="11" max="11" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="31.83203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="65" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="65"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>273</v>
       </c>
@@ -2874,23 +2874,23 @@
       <c r="H2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="J2" s="66" t="s">
+      <c r="J2" s="30" t="s">
         <v>287</v>
       </c>
-      <c r="K2" s="66" t="s">
+      <c r="K2" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="L2" s="66" t="s">
+      <c r="L2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="M2" s="66" t="s">
+      <c r="M2" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="29" customFormat="1" ht="79" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" s="29" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>277</v>
       </c>
@@ -2943,37 +2943,37 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3095ABFC-6E7C-4A65-8041-98A726BAA89B}">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.15234375" customWidth="1"/>
-    <col min="3" max="3" width="7.765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.765625" customWidth="1"/>
-    <col min="7" max="7" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.84375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.4609375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.23046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.1640625" customWidth="1"/>
+    <col min="3" max="3" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.83203125" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="65" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>273</v>
       </c>
@@ -2986,33 +2986,33 @@
       <c r="D2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="E2" s="66" t="s">
+      <c r="E2" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="30" t="s">
         <v>287</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="J2" s="66" t="s">
+      <c r="J2" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>288</v>
       </c>
       <c r="B3" s="3">
         <v>0</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="31" t="s">
         <v>132</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -3037,7 +3037,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>292</v>
       </c>
@@ -3054,37 +3054,37 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F63EA65-5E32-4F80-8A52-511467DF98D6}">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="27.23046875" customWidth="1"/>
-    <col min="4" max="4" width="25.4609375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.84375" customWidth="1"/>
-    <col min="8" max="8" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.23046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.1640625" customWidth="1"/>
+    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.83203125" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="65" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>273</v>
       </c>
@@ -3100,23 +3100,23 @@
       <c r="E2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="30" t="s">
         <v>287</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="J2" s="66" t="s">
+      <c r="J2" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>295</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>296</v>
       </c>
@@ -3165,35 +3165,35 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{821EB54D-7759-414B-B3FD-EBFB8C6B1EA5}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.23046875" customWidth="1"/>
-    <col min="3" max="5" width="12.69140625" customWidth="1"/>
-    <col min="6" max="6" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.69140625" customWidth="1"/>
-    <col min="11" max="11" width="12.23046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.1640625" customWidth="1"/>
+    <col min="3" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.6640625" customWidth="1"/>
+    <col min="11" max="11" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="65" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>273</v>
       </c>
@@ -3212,23 +3212,23 @@
       <c r="F2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="30" t="s">
         <v>287</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="J2" s="66" t="s">
+      <c r="J2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="K2" s="66" t="s">
+      <c r="K2" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="56.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>297</v>
       </c>
@@ -3275,37 +3275,37 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4D4EAF-C13B-41AE-8854-FEA63A3F8E5F}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.07421875" customWidth="1"/>
-    <col min="3" max="3" width="35.23046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.4609375" customWidth="1"/>
-    <col min="5" max="5" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="3.921875" customWidth="1"/>
-    <col min="8" max="8" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.23046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
+    <col min="3" max="3" width="35.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="65" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>273</v>
       </c>
@@ -3321,23 +3321,23 @@
       <c r="E2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="30" t="s">
         <v>287</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="J2" s="66" t="s">
+      <c r="J2" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>299</v>
       </c>
@@ -3381,35 +3381,35 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A879C41-52EB-4131-9A00-AA2D596C0624}">
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.3828125" customWidth="1"/>
-    <col min="3" max="3" width="28.84375" customWidth="1"/>
-    <col min="4" max="4" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.84375" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.83203125" customWidth="1"/>
     <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="7" max="7" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.23046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="65" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>273</v>
       </c>
@@ -3422,23 +3422,23 @@
       <c r="D2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="E2" s="66" t="s">
+      <c r="E2" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="30" t="s">
         <v>287</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>303</v>
       </c>
@@ -3479,34 +3479,34 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{449717AD-6BD6-48CE-97B0-6F3B15468816}">
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="4.765625" customWidth="1"/>
-    <col min="3" max="3" width="40.23046875" customWidth="1"/>
-    <col min="4" max="4" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.765625" customWidth="1"/>
-    <col min="7" max="7" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.23046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="4.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.1640625" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.83203125" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="65" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="33" t="s">
         <v>272</v>
       </c>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>273</v>
       </c>
@@ -3519,23 +3519,23 @@
       <c r="D2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="E2" s="66" t="s">
+      <c r="E2" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="F2" s="66" t="s">
+      <c r="F2" s="30" t="s">
         <v>287</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="I2" s="66" t="s">
+      <c r="I2" s="30" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="139.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="153" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>305</v>
       </c>
@@ -3576,40 +3576,40 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16746B8C-6F47-4FE9-9DF8-42474ABD0EFB}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.23046875" customWidth="1"/>
-    <col min="2" max="2" width="5.765625" customWidth="1"/>
-    <col min="3" max="3" width="18.61328125" customWidth="1"/>
-    <col min="4" max="4" width="30.765625" customWidth="1"/>
-    <col min="5" max="5" width="6.84375" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" customWidth="1"/>
+    <col min="2" max="2" width="5.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="6.83203125" customWidth="1"/>
     <col min="6" max="6" width="5" customWidth="1"/>
-    <col min="7" max="7" width="7.4609375" customWidth="1"/>
-    <col min="8" max="8" width="5.23046875" customWidth="1"/>
-    <col min="9" max="9" width="15.4609375" customWidth="1"/>
-    <col min="10" max="10" width="25.15234375" customWidth="1"/>
+    <col min="7" max="7" width="7.5" customWidth="1"/>
+    <col min="8" max="8" width="5.1640625" customWidth="1"/>
+    <col min="9" max="9" width="15.5" customWidth="1"/>
+    <col min="10" max="10" width="25.1640625" customWidth="1"/>
     <col min="11" max="11" width="9" customWidth="1"/>
-    <col min="12" max="14" width="2.84375" customWidth="1"/>
+    <col min="12" max="14" width="2.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="35" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="37"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="40"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3644,7 +3644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>144</v>
       </c>
@@ -3679,7 +3679,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>144</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>144</v>
       </c>
@@ -3749,7 +3749,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>144</v>
       </c>
@@ -3784,7 +3784,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>144</v>
       </c>
@@ -3819,7 +3819,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>144</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>144</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>144</v>
       </c>
@@ -3924,7 +3924,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>144</v>
       </c>
@@ -3972,41 +3972,41 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{764993EF-8B30-418C-801C-38773AF6FEE3}">
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.84375" customWidth="1"/>
-    <col min="2" max="2" width="4.15234375" customWidth="1"/>
-    <col min="3" max="3" width="10.765625" customWidth="1"/>
-    <col min="4" max="4" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.23046875" customWidth="1"/>
-    <col min="6" max="6" width="13.84375" customWidth="1"/>
-    <col min="7" max="7" width="4.765625" customWidth="1"/>
-    <col min="8" max="8" width="10.23046875" customWidth="1"/>
-    <col min="9" max="9" width="12.4609375" customWidth="1"/>
-    <col min="10" max="10" width="12.23046875" customWidth="1"/>
-    <col min="11" max="11" width="20.3828125" customWidth="1"/>
-    <col min="12" max="12" width="10.4609375" customWidth="1"/>
+    <col min="1" max="1" width="4.83203125" customWidth="1"/>
+    <col min="2" max="2" width="4.1640625" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.1640625" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="4.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.1640625" customWidth="1"/>
+    <col min="9" max="9" width="12.5" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" customWidth="1"/>
+    <col min="11" max="11" width="20.33203125" customWidth="1"/>
+    <col min="12" max="12" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="35" t="s">
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="37"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="40"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>223</v>
       </c>
@@ -4082,7 +4082,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E4">
         <v>0</v>
       </c>
@@ -4115,42 +4115,42 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{830530FE-75D5-448E-B90B-D8176BF33925}">
   <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.3828125" customWidth="1"/>
-    <col min="2" max="2" width="4.4609375" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" customWidth="1"/>
+    <col min="2" max="2" width="4.5" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="21.23046875" customWidth="1"/>
-    <col min="5" max="6" width="6.3828125" customWidth="1"/>
-    <col min="7" max="7" width="4.61328125" customWidth="1"/>
-    <col min="8" max="8" width="5.53515625" customWidth="1"/>
-    <col min="9" max="9" width="11.15234375" customWidth="1"/>
-    <col min="10" max="10" width="10.84375" customWidth="1"/>
+    <col min="4" max="4" width="21.1640625" customWidth="1"/>
+    <col min="5" max="6" width="6.33203125" customWidth="1"/>
+    <col min="7" max="7" width="4.6640625" customWidth="1"/>
+    <col min="8" max="8" width="5.5" customWidth="1"/>
+    <col min="9" max="9" width="11.1640625" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="10.84375" customWidth="1"/>
-    <col min="13" max="13" width="10.15234375" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="35" t="s">
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="37"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="40"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4191,114 +4191,114 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="48" t="s">
+    <row r="3" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="51" t="s">
         <v>215</v>
       </c>
-      <c r="B3" s="48">
+      <c r="B3" s="51">
         <v>2</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="44" t="s">
         <v>266</v>
       </c>
-      <c r="E3" s="48" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="48" t="s">
+      <c r="E3" s="51" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="51" t="s">
         <v>215</v>
       </c>
-      <c r="G3" s="48">
-        <v>7</v>
-      </c>
-      <c r="H3" s="51" t="s">
+      <c r="G3" s="51">
+        <v>7</v>
+      </c>
+      <c r="H3" s="54" t="s">
         <v>255</v>
       </c>
-      <c r="I3" s="42" t="s">
+      <c r="I3" s="45" t="s">
         <v>216</v>
       </c>
-      <c r="J3" s="45" t="s">
+      <c r="J3" s="48" t="s">
         <v>217</v>
       </c>
-      <c r="K3" s="45" t="s">
+      <c r="K3" s="48" t="s">
         <v>218</v>
       </c>
-      <c r="L3" s="45" t="s">
+      <c r="L3" s="48" t="s">
         <v>219</v>
       </c>
-      <c r="M3" s="48" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="49"/>
-      <c r="B4" s="49"/>
+      <c r="M3" s="51" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="52"/>
+      <c r="B4" s="52"/>
       <c r="C4" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="D4" s="41"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="43"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="49"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="49"/>
-      <c r="B5" s="49"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
+      <c r="M4" s="52"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="52"/>
+      <c r="B5" s="52"/>
       <c r="C5" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="D5" s="41"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="46"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="46"/>
-      <c r="M5" s="49"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="50"/>
-      <c r="B6" s="50"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="55"/>
+      <c r="I5" s="46"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+      <c r="L5" s="49"/>
+      <c r="M5" s="52"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="53"/>
+      <c r="B6" s="53"/>
       <c r="C6" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="D6" s="41"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="44"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="50"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="D6" s="44"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="50"/>
+      <c r="K6" s="50"/>
+      <c r="L6" s="50"/>
+      <c r="M6" s="53"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="H8" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="H9" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="H10" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="H11" t="s">
         <v>254</v>
       </c>
@@ -4328,35 +4328,35 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB63F1A1-E664-4B87-A4FE-643C4F1478BD}">
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.61328125" customWidth="1"/>
-    <col min="3" max="3" width="14.4609375" customWidth="1"/>
-    <col min="4" max="4" width="10.23046875" customWidth="1"/>
-    <col min="5" max="5" width="7.61328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="10.1640625" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="7" max="7" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.3828125" customWidth="1"/>
-    <col min="9" max="9" width="9.84375" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="35" t="s">
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="37"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="40"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>224</v>
       </c>
@@ -4427,41 +4427,41 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98AD8306-9A3F-48CC-80DF-BF61D33BEA56}">
   <dimension ref="A1:K32"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.4609375" customWidth="1"/>
-    <col min="3" max="3" width="9.3828125" customWidth="1"/>
-    <col min="4" max="4" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.15234375" customWidth="1"/>
-    <col min="7" max="7" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.61328125" customWidth="1"/>
-    <col min="9" max="9" width="13.84375" customWidth="1"/>
-    <col min="10" max="10" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.4609375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.5" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.1640625" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="55" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="54" t="s">
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="57" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4492,9 +4492,9 @@
       <c r="J2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="54"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K2" s="57"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>168</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>168</v>
       </c>
@@ -4564,7 +4564,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>168</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>168</v>
       </c>
@@ -4634,7 +4634,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>168</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>168</v>
       </c>
@@ -4704,7 +4704,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>168</v>
       </c>
@@ -4739,7 +4739,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>168</v>
       </c>
@@ -4774,7 +4774,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>168</v>
       </c>
@@ -4809,7 +4809,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>168</v>
       </c>
@@ -4844,7 +4844,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>168</v>
       </c>
@@ -4879,7 +4879,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>168</v>
       </c>
@@ -4914,7 +4914,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>168</v>
       </c>
@@ -4949,7 +4949,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>168</v>
       </c>
@@ -4984,7 +4984,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>168</v>
       </c>
@@ -5019,7 +5019,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>168</v>
       </c>
@@ -5054,7 +5054,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>168</v>
       </c>
@@ -5089,7 +5089,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>168</v>
       </c>
@@ -5124,7 +5124,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>168</v>
       </c>
@@ -5159,7 +5159,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>168</v>
       </c>
@@ -5194,7 +5194,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>168</v>
       </c>
@@ -5229,7 +5229,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>168</v>
       </c>
@@ -5264,7 +5264,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>168</v>
       </c>
@@ -5299,7 +5299,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>168</v>
       </c>
@@ -5334,7 +5334,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>168</v>
       </c>
@@ -5369,7 +5369,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>168</v>
       </c>
@@ -5404,7 +5404,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>168</v>
       </c>
@@ -5439,7 +5439,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>168</v>
       </c>
@@ -5474,7 +5474,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>168</v>
       </c>
@@ -5509,7 +5509,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>168</v>
       </c>
@@ -5558,39 +5558,39 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDABB22-0583-47C8-8714-261C4ED2F6DD}">
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.84375" customWidth="1"/>
-    <col min="3" max="3" width="7.23046875" customWidth="1"/>
-    <col min="4" max="4" width="19.23046875" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="7.61328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.4609375" customWidth="1"/>
-    <col min="8" max="8" width="6.15234375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.23046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="34.4609375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.83203125" customWidth="1"/>
+    <col min="3" max="3" width="7.1640625" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="35" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="54" t="s">
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="57" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -5618,9 +5618,9 @@
       <c r="I2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="54"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="J2" s="57"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>169</v>
       </c>
@@ -5652,7 +5652,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>169</v>
       </c>
@@ -5684,7 +5684,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>169</v>
       </c>
@@ -5716,7 +5716,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>169</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>169</v>
       </c>
@@ -5780,7 +5780,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>169</v>
       </c>
@@ -5812,7 +5812,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>169</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>169</v>
       </c>
@@ -5876,7 +5876,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>169</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>169</v>
       </c>
@@ -5940,7 +5940,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>169</v>
       </c>
@@ -5972,7 +5972,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>169</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>169</v>
       </c>
@@ -6036,7 +6036,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>169</v>
       </c>
@@ -6068,7 +6068,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>169</v>
       </c>
@@ -6100,7 +6100,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>169</v>
       </c>
@@ -6132,7 +6132,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>169</v>
       </c>
@@ -6164,7 +6164,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>169</v>
       </c>
@@ -6196,7 +6196,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>169</v>
       </c>
@@ -6228,7 +6228,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>169</v>
       </c>
@@ -6260,7 +6260,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>169</v>
       </c>
@@ -6292,7 +6292,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>169</v>
       </c>
@@ -6324,7 +6324,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>169</v>
       </c>
@@ -6356,7 +6356,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>169</v>
       </c>
@@ -6388,7 +6388,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>169</v>
       </c>
@@ -6420,7 +6420,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>169</v>
       </c>
@@ -6452,7 +6452,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>169</v>
       </c>
@@ -6484,7 +6484,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>169</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>169</v>
       </c>
@@ -6548,7 +6548,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>169</v>
       </c>
@@ -6594,47 +6594,47 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ADC9217-D3D6-4678-A1D4-C4F96C78FB27}">
   <dimension ref="A1:L34"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" style="23" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" style="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" style="23" customWidth="1"/>
     <col min="3" max="3" width="10" style="23" customWidth="1"/>
-    <col min="4" max="4" width="9.15234375" style="23" customWidth="1"/>
-    <col min="5" max="5" width="6.15234375" style="23" customWidth="1"/>
-    <col min="6" max="6" width="5.765625" style="23" customWidth="1"/>
-    <col min="7" max="7" width="6.15234375" style="23" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1640625" style="23" customWidth="1"/>
+    <col min="5" max="5" width="6.1640625" style="23" customWidth="1"/>
+    <col min="6" max="6" width="5.83203125" style="23" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" style="23" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="23" customWidth="1"/>
-    <col min="9" max="9" width="16.4609375" style="23" customWidth="1"/>
-    <col min="10" max="10" width="9.84375" style="23" customWidth="1"/>
-    <col min="11" max="11" width="27.61328125" style="23" customWidth="1"/>
-    <col min="12" max="12" width="31.15234375" style="23" customWidth="1"/>
-    <col min="13" max="14" width="3.15234375" style="23" customWidth="1"/>
+    <col min="9" max="9" width="16.5" style="23" customWidth="1"/>
+    <col min="10" max="10" width="9.83203125" style="23" customWidth="1"/>
+    <col min="11" max="11" width="27.6640625" style="23" customWidth="1"/>
+    <col min="12" max="12" width="31.1640625" style="23" customWidth="1"/>
+    <col min="13" max="14" width="3.1640625" style="23" customWidth="1"/>
     <col min="15" max="16384" width="9" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="58" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="57" t="s">
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="60" t="s">
         <v>191</v>
       </c>
-      <c r="L1" s="56" t="s">
+      <c r="L1" s="59" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
@@ -6665,10 +6665,10 @@
       <c r="J2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
@@ -6706,7 +6706,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
         <v>2</v>
       </c>
@@ -6744,7 +6744,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
         <v>2</v>
       </c>
@@ -6782,7 +6782,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
         <v>2</v>
       </c>
@@ -6820,7 +6820,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
         <v>2</v>
       </c>
@@ -6858,7 +6858,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
         <v>2</v>
       </c>
@@ -6896,7 +6896,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
         <v>2</v>
       </c>
@@ -6934,7 +6934,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>2</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
         <v>2</v>
       </c>
@@ -7010,7 +7010,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
         <v>2</v>
       </c>
@@ -7048,7 +7048,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>2</v>
       </c>
@@ -7086,7 +7086,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
         <v>2</v>
       </c>
@@ -7124,7 +7124,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="21" t="s">
         <v>2</v>
       </c>
@@ -7159,7 +7159,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
         <v>2</v>
       </c>
@@ -7194,7 +7194,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="21" t="s">
         <v>2</v>
       </c>
@@ -7229,7 +7229,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="21" t="s">
         <v>2</v>
       </c>
@@ -7264,7 +7264,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="21" t="s">
         <v>2</v>
       </c>
@@ -7299,7 +7299,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="21" t="s">
         <v>2</v>
       </c>
@@ -7334,7 +7334,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
         <v>2</v>
       </c>
@@ -7369,7 +7369,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="20" t="s">
         <v>2</v>
       </c>
@@ -7407,7 +7407,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
         <v>2</v>
       </c>
@@ -7445,7 +7445,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="20" t="s">
         <v>2</v>
       </c>
@@ -7483,7 +7483,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="20" t="s">
         <v>2</v>
       </c>
@@ -7521,7 +7521,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="20" t="s">
         <v>2</v>
       </c>
@@ -7559,7 +7559,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="20" t="s">
         <v>2</v>
       </c>
@@ -7597,7 +7597,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="20" t="s">
         <v>2</v>
       </c>
@@ -7635,7 +7635,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
         <v>2</v>
       </c>
@@ -7673,7 +7673,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
         <v>2</v>
       </c>
@@ -7711,7 +7711,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="20" t="s">
         <v>2</v>
       </c>
@@ -7749,7 +7749,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="20" t="s">
         <v>2</v>
       </c>
@@ -7787,7 +7787,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="20" t="s">
         <v>2</v>
       </c>
@@ -7825,7 +7825,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="L34" s="24"/>
     </row>
   </sheetData>
@@ -7843,45 +7843,45 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22D51970-3AD2-45D3-AAEB-95AEA9D3D696}">
   <dimension ref="A1:K33"/>
-  <sheetFormatPr defaultColWidth="9.23046875" defaultRowHeight="16" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.61328125" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.15234375" style="9" customWidth="1"/>
-    <col min="3" max="3" width="11.15234375" style="9" customWidth="1"/>
-    <col min="4" max="4" width="7.84375" style="9" customWidth="1"/>
-    <col min="5" max="5" width="9.23046875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="7.61328125" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.23046875" style="9" customWidth="1"/>
-    <col min="8" max="8" width="6.15234375" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.84375" style="9" customWidth="1"/>
-    <col min="10" max="10" width="27.4609375" style="9" customWidth="1"/>
-    <col min="11" max="11" width="31.15234375" style="9" customWidth="1"/>
-    <col min="12" max="13" width="2.4609375" style="9" customWidth="1"/>
-    <col min="14" max="16384" width="9.23046875" style="9"/>
+    <col min="1" max="1" width="7.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.1640625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="9.1640625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.1640625" style="9" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.83203125" style="9" customWidth="1"/>
+    <col min="10" max="10" width="27.5" style="9" customWidth="1"/>
+    <col min="11" max="11" width="31.1640625" style="9" customWidth="1"/>
+    <col min="12" max="13" width="2.5" style="9" customWidth="1"/>
+    <col min="14" max="16384" width="9.1640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A1" s="59" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="31" t="s">
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="57" t="s">
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="60" t="s">
         <v>191</v>
       </c>
-      <c r="K1" s="56" t="s">
+      <c r="K1" s="59" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
@@ -7909,10 +7909,10 @@
       <c r="I2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>170</v>
       </c>
@@ -7947,7 +7947,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
         <v>170</v>
       </c>
@@ -7982,7 +7982,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
         <v>170</v>
       </c>
@@ -8017,7 +8017,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
         <v>170</v>
       </c>
@@ -8052,7 +8052,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
         <v>170</v>
       </c>
@@ -8087,7 +8087,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
         <v>170</v>
       </c>
@@ -8122,7 +8122,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
         <v>170</v>
       </c>
@@ -8157,7 +8157,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>170</v>
       </c>
@@ -8192,7 +8192,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
         <v>170</v>
       </c>
@@ -8227,7 +8227,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
         <v>170</v>
       </c>
@@ -8262,7 +8262,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>170</v>
       </c>
@@ -8297,7 +8297,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
         <v>170</v>
       </c>
@@ -8332,7 +8332,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="21" t="s">
         <v>170</v>
       </c>
@@ -8360,12 +8360,12 @@
       <c r="I15" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="J15" s="62"/>
+      <c r="J15" s="65"/>
       <c r="K15" s="21" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
         <v>170</v>
       </c>
@@ -8393,12 +8393,12 @@
       <c r="I16" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="J16" s="63"/>
+      <c r="J16" s="66"/>
       <c r="K16" s="21" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="21" t="s">
         <v>170</v>
       </c>
@@ -8426,12 +8426,12 @@
       <c r="I17" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="J17" s="63"/>
+      <c r="J17" s="66"/>
       <c r="K17" s="21" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="21" t="s">
         <v>170</v>
       </c>
@@ -8459,12 +8459,12 @@
       <c r="I18" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="J18" s="63"/>
+      <c r="J18" s="66"/>
       <c r="K18" s="21" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="21" t="s">
         <v>170</v>
       </c>
@@ -8492,12 +8492,12 @@
       <c r="I19" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="J19" s="63"/>
+      <c r="J19" s="66"/>
       <c r="K19" s="21" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="21" t="s">
         <v>170</v>
       </c>
@@ -8525,12 +8525,12 @@
       <c r="I20" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="J20" s="63"/>
+      <c r="J20" s="66"/>
       <c r="K20" s="21" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
         <v>170</v>
       </c>
@@ -8558,12 +8558,12 @@
       <c r="I21" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="J21" s="64"/>
+      <c r="J21" s="67"/>
       <c r="K21" s="21" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="20" t="s">
         <v>170</v>
       </c>
@@ -8598,7 +8598,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
         <v>170</v>
       </c>
@@ -8633,7 +8633,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="20" t="s">
         <v>170</v>
       </c>
@@ -8668,7 +8668,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="20" t="s">
         <v>170</v>
       </c>
@@ -8703,7 +8703,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="20" t="s">
         <v>170</v>
       </c>
@@ -8738,7 +8738,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="20" t="s">
         <v>170</v>
       </c>
@@ -8773,7 +8773,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="20" t="s">
         <v>170</v>
       </c>
@@ -8808,7 +8808,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
         <v>170</v>
       </c>
@@ -8843,7 +8843,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
         <v>170</v>
       </c>
@@ -8878,7 +8878,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="20" t="s">
         <v>170</v>
       </c>
@@ -8913,7 +8913,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="20" t="s">
         <v>170</v>
       </c>
@@ -8948,7 +8948,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="20" t="s">
         <v>170</v>
       </c>

</xml_diff>